<commit_message>
fix: narrow Excel template to New-Report-only, drop RecordType/Cancel
</commit_message>
<xml_diff>
--- a/mikadiv-vib/generated/mikadiv-vib-v1.0.0.xlsx
+++ b/mikadiv-vib/generated/mikadiv-vib-v1.0.0.xlsx
@@ -530,7 +530,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B28"/>
+  <dimension ref="A1:B27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="42" customWidth="1" min="1" max="1"/>
@@ -685,129 +685,117 @@
       </c>
       <c r="B16" s="4" t="inlineStr">
         <is>
-          <t>The key on '1 Requests Master' and the first column on every other sheet. It is only used to link the sheets, so any unique value works (it does not need to be a UUID). Use the same RequestId to join a request's data across all sheets.</t>
+          <t>The key on '1 Requests Master' and the first column on every other sheet, used to join a request's data across all sheets. Per VIB's own schema, RequestId must stay unique even across files you submit later, not just within this one -- corrections and cancellations you submit afterward reference it by exact value.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="5" t="inlineStr">
-        <is>
-          <t>Request vs Cancel</t>
-        </is>
-      </c>
-      <c r="B17" s="4" t="inlineStr">
-        <is>
-          <t>Set RecordType on '1 Requests Master'. For 'Cancel' rows, fill PreviousRequestIdForCancellation (and optionally ReportSerialNumber) and leave all other sheets empty for that RequestId.</t>
-        </is>
-      </c>
+      <c r="A17" s="5" t="inlineStr"/>
+      <c r="B17" s="4" t="inlineStr"/>
     </row>
     <row r="18">
-      <c r="A18" s="5" t="inlineStr"/>
+      <c r="A18" s="3" t="inlineStr">
+        <is>
+          <t>Cardinality (rows per RequestId)</t>
+        </is>
+      </c>
       <c r="B18" s="4" t="inlineStr"/>
     </row>
     <row r="19">
-      <c r="A19" s="3" t="inlineStr">
-        <is>
-          <t>Cardinality (rows per RequestId)</t>
-        </is>
-      </c>
-      <c r="B19" s="4" t="inlineStr"/>
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>2 Security Related Information</t>
+        </is>
+      </c>
+      <c r="B19" s="4" t="inlineStr">
+        <is>
+          <t>0..1 (required for Request records). Includes the depositary-receipt fields, which are required when IsDepositaryReceipt = true.</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="5" t="inlineStr">
         <is>
-          <t>2 Security Related Information</t>
+          <t>3 Tax Voucher Individuals / 4 Tax Voucher Legal Persons</t>
         </is>
       </c>
       <c r="B20" s="4" t="inlineStr">
         <is>
-          <t>0..1 (required for Request records). Includes the depositary-receipt fields, which are required when IsDepositaryReceipt = true.</t>
+          <t>Tax voucher receivers: up to 2 receivers in total per request (across both sheets).</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>3 Tax Voucher Individuals / 4 Tax Voucher Legal Persons</t>
+          <t>5 Third Party Individuals / 6 Third Party Legal Persons</t>
         </is>
       </c>
       <c r="B21" s="4" t="inlineStr">
         <is>
-          <t>Tax voucher receivers: up to 2 receivers in total per request (across both sheets).</t>
+          <t>Third-party owners: up to 5 in total per request (across both sheets).</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>5 Third Party Individuals / 6 Third Party Legal Persons</t>
+          <t>7 Custody Chain</t>
         </is>
       </c>
       <c r="B22" s="4" t="inlineStr">
         <is>
-          <t>Third-party owners: up to 5 in total per request (across both sheets).</t>
+          <t>Up to 20 links per request; sort by NumberInChain (1 = closest to the beneficiary).</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>7 Custody Chain</t>
+          <t>8 FIFO Trades</t>
         </is>
       </c>
       <c r="B23" s="4" t="inlineStr">
         <is>
-          <t>Up to 20 links per request; sort by NumberInChain (1 = closest to the beneficiary).</t>
+          <t>Up to 1000 Receipt rows and 1000 Delivery rows per request (use when ReceiptsAndDeliveriesMode = FiFo).</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="5" t="inlineStr">
         <is>
-          <t>8 FIFO Trades</t>
+          <t>9 Raw Transactions All</t>
         </is>
       </c>
       <c r="B24" s="4" t="inlineStr">
         <is>
-          <t>Up to 1000 Receipt rows and 1000 Delivery rows per request (use when ReceiptsAndDeliveriesMode = FiFo).</t>
+          <t>Unbounded rows per request (use when ReceiptsAndDeliveriesMode = All).</t>
         </is>
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
-        <is>
-          <t>9 Raw Transactions All</t>
-        </is>
-      </c>
-      <c r="B25" s="4" t="inlineStr">
-        <is>
-          <t>Unbounded rows per request (use when ReceiptsAndDeliveriesMode = All).</t>
-        </is>
-      </c>
+      <c r="A25" s="5" t="inlineStr"/>
+      <c r="B25" s="4" t="inlineStr"/>
     </row>
     <row r="26">
-      <c r="A26" s="5" t="inlineStr"/>
-      <c r="B26" s="4" t="inlineStr"/>
+      <c r="A26" s="5" t="inlineStr">
+        <is>
+          <t>Community recipients</t>
+        </is>
+      </c>
+      <c r="B26" s="4" t="inlineStr">
+        <is>
+          <t>A community tax certificate receiver (up to 10 members) is captured by setting ReceiverGroupType = CommunityMember on the tax voucher sheets and giving all members of one community the same CommunityGroupId.</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>Community recipients</t>
+          <t>Enum dropdowns</t>
         </is>
       </c>
       <c r="B27" s="4" t="inlineStr">
-        <is>
-          <t>A community tax certificate receiver (up to 10 members) is captured by setting ReceiverGroupType = CommunityMember on the tax voucher sheets and giving all members of one community the same CommunityGroupId.</t>
-        </is>
-      </c>
-    </row>
-    <row r="28">
-      <c r="A28" s="5" t="inlineStr">
-        <is>
-          <t>Enum dropdowns</t>
-        </is>
-      </c>
-      <c r="B28" s="4" t="inlineStr">
         <is>
           <t>Cells backed by a fixed value list provide an in-cell dropdown. Manual values outside the list are rejected.</t>
         </is>
@@ -1142,34 +1130,32 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y4"/>
+  <dimension ref="A1:W4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
     <col width="18" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="26" customWidth="1" min="5" max="5"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
+    <col width="27" customWidth="1" min="5" max="5"/>
     <col width="27" customWidth="1" min="6" max="6"/>
-    <col width="27" customWidth="1" min="7" max="7"/>
-    <col width="19" customWidth="1" min="8" max="8"/>
-    <col width="25" customWidth="1" min="9" max="9"/>
-    <col width="27" customWidth="1" min="10" max="10"/>
-    <col width="22" customWidth="1" min="11" max="11"/>
-    <col width="33" customWidth="1" min="12" max="12"/>
-    <col width="21" customWidth="1" min="13" max="13"/>
-    <col width="41" customWidth="1" min="14" max="14"/>
+    <col width="19" customWidth="1" min="7" max="7"/>
+    <col width="25" customWidth="1" min="8" max="8"/>
+    <col width="27" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="33" customWidth="1" min="11" max="11"/>
+    <col width="21" customWidth="1" min="12" max="12"/>
+    <col width="41" customWidth="1" min="13" max="13"/>
+    <col width="42" customWidth="1" min="14" max="14"/>
     <col width="42" customWidth="1" min="15" max="15"/>
-    <col width="42" customWidth="1" min="16" max="16"/>
-    <col width="41" customWidth="1" min="17" max="17"/>
+    <col width="41" customWidth="1" min="16" max="16"/>
+    <col width="42" customWidth="1" min="17" max="17"/>
     <col width="42" customWidth="1" min="18" max="18"/>
-    <col width="42" customWidth="1" min="19" max="19"/>
+    <col width="18" customWidth="1" min="19" max="19"/>
     <col width="18" customWidth="1" min="20" max="20"/>
-    <col width="18" customWidth="1" min="21" max="21"/>
-    <col width="35" customWidth="1" min="22" max="22"/>
-    <col width="26" customWidth="1" min="23" max="23"/>
-    <col width="18" customWidth="1" min="24" max="24"/>
-    <col width="22" customWidth="1" min="25" max="25"/>
+    <col width="26" customWidth="1" min="21" max="21"/>
+    <col width="18" customWidth="1" min="22" max="22"/>
+    <col width="22" customWidth="1" min="23" max="23"/>
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
@@ -1180,120 +1166,110 @@
       </c>
       <c r="B1" s="6" t="inlineStr">
         <is>
-          <t>RecordType</t>
+          <t>AccountNumber</t>
         </is>
       </c>
       <c r="C1" s="6" t="inlineStr">
         <is>
-          <t>AccountNumber</t>
+          <t>ClientReference</t>
         </is>
       </c>
       <c r="D1" s="6" t="inlineStr">
         <is>
-          <t>ClientReference</t>
+          <t>ClientContactpersonName</t>
         </is>
       </c>
       <c r="E1" s="6" t="inlineStr">
         <is>
-          <t>ClientContactpersonName</t>
+          <t>ClientContactpersonPhone</t>
         </is>
       </c>
       <c r="F1" s="6" t="inlineStr">
         <is>
-          <t>ClientContactpersonPhone</t>
+          <t>ClientContactpersonEmail</t>
         </is>
       </c>
       <c r="G1" s="6" t="inlineStr">
         <is>
-          <t>ClientContactpersonEmail</t>
+          <t>RequestedService</t>
         </is>
       </c>
       <c r="H1" s="6" t="inlineStr">
         <is>
-          <t>RequestedService</t>
+          <t>RequestedServiceReason</t>
         </is>
       </c>
       <c r="I1" s="6" t="inlineStr">
         <is>
-          <t>RequestedServiceReason</t>
+          <t>RequestedAttestationType</t>
         </is>
       </c>
       <c r="J1" s="6" t="inlineStr">
         <is>
-          <t>RequestedAttestationType</t>
+          <t>IsCorrectionRequest</t>
         </is>
       </c>
       <c r="K1" s="6" t="inlineStr">
         <is>
-          <t>IsCorrectionRequest</t>
+          <t>PreviousRequestIdForCorrection</t>
         </is>
       </c>
       <c r="L1" s="6" t="inlineStr">
         <is>
-          <t>PreviousRequestIdForCorrection</t>
+          <t>ReportSerialNumber</t>
         </is>
       </c>
       <c r="M1" s="6" t="inlineStr">
         <is>
-          <t>ReportSerialNumber</t>
+          <t>TaxCertificatePrintedContactpersonName</t>
         </is>
       </c>
       <c r="N1" s="6" t="inlineStr">
         <is>
-          <t>TaxCertificatePrintedContactpersonName</t>
+          <t>TaxCertificatePrintedContactpersonPhone</t>
         </is>
       </c>
       <c r="O1" s="6" t="inlineStr">
         <is>
-          <t>TaxCertificatePrintedContactpersonPhone</t>
+          <t>TaxCertificatePrintedContactpersonEmail</t>
         </is>
       </c>
       <c r="P1" s="6" t="inlineStr">
         <is>
-          <t>TaxCertificatePrintedContactpersonEmail</t>
+          <t>TaxCertificateAlternativeRecipientName</t>
         </is>
       </c>
       <c r="Q1" s="6" t="inlineStr">
         <is>
-          <t>TaxCertificateAlternativeRecipientName</t>
+          <t>TaxCertificateAlternativeRecipientAddress</t>
         </is>
       </c>
       <c r="R1" s="6" t="inlineStr">
         <is>
-          <t>TaxCertificateAlternativeRecipientAddress</t>
+          <t>TaxCertificateAlternativeRecipientEmail</t>
         </is>
       </c>
       <c r="S1" s="6" t="inlineStr">
         <is>
-          <t>TaxCertificateAlternativeRecipientEmail</t>
+          <t>EventType</t>
         </is>
       </c>
       <c r="T1" s="6" t="inlineStr">
         <is>
-          <t>EventType</t>
+          <t>FundId</t>
         </is>
       </c>
       <c r="U1" s="6" t="inlineStr">
         <is>
-          <t>FundId</t>
+          <t>SecuritiesAccountNumber</t>
         </is>
       </c>
       <c r="V1" s="6" t="inlineStr">
         <is>
-          <t>PreviousRequestIdForCancellation</t>
+          <t>AccountType</t>
         </is>
       </c>
       <c r="W1" s="6" t="inlineStr">
-        <is>
-          <t>SecuritiesAccountNumber</t>
-        </is>
-      </c>
-      <c r="X1" s="6" t="inlineStr">
-        <is>
-          <t>AccountType</t>
-        </is>
-      </c>
-      <c r="Y1" s="6" t="inlineStr">
         <is>
           <t>AccountRelationship</t>
         </is>
@@ -1307,120 +1283,110 @@
       </c>
       <c r="B2" s="7" t="inlineStr">
         <is>
-          <t>'Request' for a MiKaDiv reporting for income; 'Cancel' to cancel a previously submitted request (leave the child sheets empty for cancellation rows).</t>
+          <t>Account number of the requesting custodian.</t>
         </is>
       </c>
       <c r="C2" s="7" t="inlineStr">
         <is>
-          <t>Account number of the requesting custodian.</t>
+          <t>Custom reference data of the client.</t>
         </is>
       </c>
       <c r="D2" s="7" t="inlineStr">
         <is>
-          <t>Custom reference data of the client.</t>
+          <t>Name of the responsible foreign bank contact person.</t>
         </is>
       </c>
       <c r="E2" s="7" t="inlineStr">
         <is>
-          <t>Name of the responsible foreign bank contact person.</t>
+          <t>Telephone number of the responsible foreign bank contact person.</t>
         </is>
       </c>
       <c r="F2" s="7" t="inlineStr">
         <is>
-          <t>Telephone number of the responsible foreign bank contact person.</t>
+          <t>E-mail address of the responsible foreign bank contact person.</t>
         </is>
       </c>
       <c r="G2" s="7" t="inlineStr">
         <is>
-          <t>E-mail address of the responsible foreign bank contact person.</t>
+          <t>Type of requested service.</t>
         </is>
       </c>
       <c r="H2" s="7" t="inlineStr">
         <is>
-          <t>Type of requested service.</t>
+          <t>Reason for the requested service, especially for correction or cancellation.</t>
         </is>
       </c>
       <c r="I2" s="7" t="inlineStr">
         <is>
-          <t>Reason for the requested service, especially for correction or cancellation.</t>
+          <t>Type of requested tax voucher.</t>
         </is>
       </c>
       <c r="J2" s="7" t="inlineStr">
         <is>
-          <t>Type of requested tax voucher.</t>
+          <t>A correction is to be performed for a report. The data record contains a reference to the preceding request.</t>
         </is>
       </c>
       <c r="K2" s="7" t="inlineStr">
         <is>
-          <t>A correction is to be performed for a report. The data record contains a reference to the preceding request.</t>
+          <t>If the request is for correction of a previous request, then the RequestId of the previous request must be provided.</t>
         </is>
       </c>
       <c r="L2" s="7" t="inlineStr">
         <is>
-          <t>If the request is for correction of a previous request, then the RequestId of the previous request must be provided.</t>
+          <t>Serial number (UUID) of an already submitted report, if provided previously by the German Paying agent. Used as a (additional) reference for correction.</t>
         </is>
       </c>
       <c r="M2" s="7" t="inlineStr">
         <is>
-          <t>Serial number (UUID) of an already submitted report, if provided previously by the German Paying agent. Used as a (additional) reference for correction.</t>
+          <t>Name of the contact person for the customer, printed on the tax certificate or cover letter.</t>
         </is>
       </c>
       <c r="N2" s="7" t="inlineStr">
         <is>
-          <t>Name of the contact person for the customer, printed on the tax certificate or cover letter.</t>
+          <t>Telephone number of the contact person for the customer, printed on the tax certificate or cover letter.</t>
         </is>
       </c>
       <c r="O2" s="7" t="inlineStr">
         <is>
-          <t>Telephone number of the contact person for the customer, printed on the tax certificate or cover letter.</t>
+          <t>E-mail address of the contact person for the customer, printed on the tax certificate or cover letter.</t>
         </is>
       </c>
       <c r="P2" s="7" t="inlineStr">
         <is>
-          <t>E-mail address of the contact person for the customer, printed on the tax certificate or cover letter.</t>
+          <t>Name of the alternative mailing address recipient.</t>
         </is>
       </c>
       <c r="Q2" s="7" t="inlineStr">
         <is>
-          <t>Name of the alternative mailing address recipient.</t>
+          <t>Address of the alternative mailing address recipient.</t>
         </is>
       </c>
       <c r="R2" s="7" t="inlineStr">
         <is>
-          <t>Address of the alternative mailing address recipient.</t>
+          <t>E-mail address of the alternative mailing address recipient.</t>
         </is>
       </c>
       <c r="S2" s="7" t="inlineStr">
         <is>
-          <t>E-mail address of the alternative mailing address recipient.</t>
+          <t>Event designations of the German paying agent according to ISO 20022.</t>
         </is>
       </c>
       <c r="T2" s="7" t="inlineStr">
         <is>
-          <t>Event designations of the German paying agent according to ISO 20022.</t>
+          <t>Fund identifier (status certificate number).</t>
         </is>
       </c>
       <c r="U2" s="7" t="inlineStr">
         <is>
-          <t>Fund identifier (status certificate number).</t>
+          <t>Account number of the tax voucher person at the custodian to whom the tax voucher person is directly contracted.</t>
         </is>
       </c>
       <c r="V2" s="7" t="inlineStr">
         <is>
-          <t>If the request is for cancellation of a previous request, then the RequestId of the previous request must be provided.</t>
+          <t>Account type.</t>
         </is>
       </c>
       <c r="W2" s="7" t="inlineStr">
-        <is>
-          <t>Account number of the tax voucher person at the custodian to whom the tax voucher person is directly contracted.</t>
-        </is>
-      </c>
-      <c r="X2" s="7" t="inlineStr">
-        <is>
-          <t>Account type.</t>
-        </is>
-      </c>
-      <c r="Y2" s="7" t="inlineStr">
         <is>
           <t>If the tax voucher person is not the beneficial owner (creditor), then the account relationship has to be specified.</t>
         </is>
@@ -1434,7 +1400,7 @@
       </c>
       <c r="B3" s="8" t="inlineStr">
         <is>
-          <t>Choose one: Request | Cancel</t>
+          <t>Text (max 200)</t>
         </is>
       </c>
       <c r="C3" s="8" t="inlineStr">
@@ -1449,105 +1415,95 @@
       </c>
       <c r="E3" s="8" t="inlineStr">
         <is>
+          <t>Text (max 35)</t>
+        </is>
+      </c>
+      <c r="F3" s="8" t="inlineStr">
+        <is>
           <t>Text (max 200)</t>
         </is>
       </c>
-      <c r="F3" s="8" t="inlineStr">
+      <c r="G3" s="8" t="inlineStr">
+        <is>
+          <t>Choose one: TaxReportAndCertificate | Reclaim | Relief</t>
+        </is>
+      </c>
+      <c r="H3" s="8" t="inlineStr">
+        <is>
+          <t>Text (max 256)</t>
+        </is>
+      </c>
+      <c r="I3" s="8" t="inlineStr">
+        <is>
+          <t>Choose one: BV | PV | SB</t>
+        </is>
+      </c>
+      <c r="J3" s="8" t="inlineStr">
+        <is>
+          <t>Choose one: true | false</t>
+        </is>
+      </c>
+      <c r="K3" s="8" t="inlineStr">
+        <is>
+          <t>UUID (xxxxxxxx-xxxx-xxxx-xxxx-xxxxxxxxxxxx)</t>
+        </is>
+      </c>
+      <c r="L3" s="8" t="inlineStr">
+        <is>
+          <t>UUID (xxxxxxxx-xxxx-xxxx-xxxx-xxxxxxxxxxxx)</t>
+        </is>
+      </c>
+      <c r="M3" s="8" t="inlineStr">
+        <is>
+          <t>Text (max 200)</t>
+        </is>
+      </c>
+      <c r="N3" s="8" t="inlineStr">
         <is>
           <t>Text (max 35)</t>
         </is>
       </c>
-      <c r="G3" s="8" t="inlineStr">
+      <c r="O3" s="8" t="inlineStr">
         <is>
           <t>Text (max 200)</t>
         </is>
       </c>
-      <c r="H3" s="8" t="inlineStr">
-        <is>
-          <t>Choose one: TaxReportAndCertificate | Reclaim | Relief</t>
-        </is>
-      </c>
-      <c r="I3" s="8" t="inlineStr">
+      <c r="P3" s="8" t="inlineStr">
+        <is>
+          <t>Text (max 200)</t>
+        </is>
+      </c>
+      <c r="Q3" s="8" t="inlineStr">
         <is>
           <t>Text (max 256)</t>
         </is>
       </c>
-      <c r="J3" s="8" t="inlineStr">
-        <is>
-          <t>Choose one: BV | PV | SB</t>
-        </is>
-      </c>
-      <c r="K3" s="8" t="inlineStr">
-        <is>
-          <t>Choose one: true | false</t>
-        </is>
-      </c>
-      <c r="L3" s="8" t="inlineStr">
-        <is>
-          <t>UUID (xxxxxxxx-xxxx-xxxx-xxxx-xxxxxxxxxxxx)</t>
-        </is>
-      </c>
-      <c r="M3" s="8" t="inlineStr">
-        <is>
-          <t>UUID (xxxxxxxx-xxxx-xxxx-xxxx-xxxxxxxxxxxx)</t>
-        </is>
-      </c>
-      <c r="N3" s="8" t="inlineStr">
+      <c r="R3" s="8" t="inlineStr">
+        <is>
+          <t>Text (max 256)</t>
+        </is>
+      </c>
+      <c r="S3" s="8" t="inlineStr">
+        <is>
+          <t>Text (max 20)</t>
+        </is>
+      </c>
+      <c r="T3" s="8" t="inlineStr">
+        <is>
+          <t>Text (max 20)</t>
+        </is>
+      </c>
+      <c r="U3" s="8" t="inlineStr">
         <is>
           <t>Text (max 200)</t>
         </is>
       </c>
-      <c r="O3" s="8" t="inlineStr">
-        <is>
-          <t>Text (max 35)</t>
-        </is>
-      </c>
-      <c r="P3" s="8" t="inlineStr">
-        <is>
-          <t>Text (max 200)</t>
-        </is>
-      </c>
-      <c r="Q3" s="8" t="inlineStr">
-        <is>
-          <t>Text (max 200)</t>
-        </is>
-      </c>
-      <c r="R3" s="8" t="inlineStr">
-        <is>
-          <t>Text (max 256)</t>
-        </is>
-      </c>
-      <c r="S3" s="8" t="inlineStr">
-        <is>
-          <t>Text (max 256)</t>
-        </is>
-      </c>
-      <c r="T3" s="8" t="inlineStr">
-        <is>
-          <t>Text (max 20)</t>
-        </is>
-      </c>
-      <c r="U3" s="8" t="inlineStr">
-        <is>
-          <t>Text (max 20)</t>
-        </is>
-      </c>
       <c r="V3" s="8" t="inlineStr">
         <is>
-          <t>UUID (xxxxxxxx-xxxx-xxxx-xxxx-xxxxxxxxxxxx)</t>
+          <t>Choose one: A | B | Ct | D | E | F | G</t>
         </is>
       </c>
       <c r="W3" s="8" t="inlineStr">
-        <is>
-          <t>Text (max 200)</t>
-        </is>
-      </c>
-      <c r="X3" s="8" t="inlineStr">
-        <is>
-          <t>Choose one: A | B | Ct | D | E | F | G</t>
-        </is>
-      </c>
-      <c r="Y3" s="8" t="inlineStr">
         <is>
           <t>Choose one: Trust | Usufruct | Pledge</t>
         </is>
@@ -1564,9 +1520,9 @@
           <t>Required</t>
         </is>
       </c>
-      <c r="C4" s="9" t="inlineStr">
-        <is>
-          <t>Required</t>
+      <c r="C4" s="10" t="inlineStr">
+        <is>
+          <t>Optional</t>
         </is>
       </c>
       <c r="D4" s="10" t="inlineStr">
@@ -1584,16 +1540,16 @@
           <t>Optional</t>
         </is>
       </c>
-      <c r="G4" s="10" t="inlineStr">
-        <is>
-          <t>Optional</t>
-        </is>
-      </c>
-      <c r="H4" s="11" t="inlineStr">
+      <c r="G4" s="11" t="inlineStr">
         <is>
           <t>Conditional</t>
         </is>
       </c>
+      <c r="H4" s="10" t="inlineStr">
+        <is>
+          <t>Optional</t>
+        </is>
+      </c>
       <c r="I4" s="10" t="inlineStr">
         <is>
           <t>Optional</t>
@@ -1654,9 +1610,9 @@
           <t>Optional</t>
         </is>
       </c>
-      <c r="U4" s="10" t="inlineStr">
-        <is>
-          <t>Optional</t>
+      <c r="U4" s="11" t="inlineStr">
+        <is>
+          <t>Conditional</t>
         </is>
       </c>
       <c r="V4" s="11" t="inlineStr">
@@ -1664,40 +1620,27 @@
           <t>Conditional</t>
         </is>
       </c>
-      <c r="W4" s="11" t="inlineStr">
-        <is>
-          <t>Conditional</t>
-        </is>
-      </c>
-      <c r="X4" s="11" t="inlineStr">
-        <is>
-          <t>Conditional</t>
-        </is>
-      </c>
-      <c r="Y4" s="10" t="inlineStr">
+      <c r="W4" s="10" t="inlineStr">
         <is>
           <t>Optional</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="6">
-    <dataValidation sqref="B5:B1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Please choose a value from the dropdown list." type="list" errorStyle="stop">
-      <formula1>"Request,Cancel"</formula1>
-    </dataValidation>
-    <dataValidation sqref="H5:H1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Please choose a value from the dropdown list." type="list" errorStyle="stop">
+  <dataValidations count="5">
+    <dataValidation sqref="G5:G1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Please choose a value from the dropdown list." type="list" errorStyle="stop">
       <formula1>"TaxReportAndCertificate,Reclaim,Relief"</formula1>
     </dataValidation>
-    <dataValidation sqref="J5:J1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Please choose a value from the dropdown list." type="list" errorStyle="stop">
+    <dataValidation sqref="I5:I1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Please choose a value from the dropdown list." type="list" errorStyle="stop">
       <formula1>"BV,PV,SB"</formula1>
     </dataValidation>
-    <dataValidation sqref="K5:K1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Please choose a value from the dropdown list." type="list" errorStyle="stop">
+    <dataValidation sqref="J5:J1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Please choose a value from the dropdown list." type="list" errorStyle="stop">
       <formula1>"true,false"</formula1>
     </dataValidation>
-    <dataValidation sqref="X5:X1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Please choose a value from the dropdown list." type="list" errorStyle="stop">
+    <dataValidation sqref="V5:V1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Please choose a value from the dropdown list." type="list" errorStyle="stop">
       <formula1>"A,B,Ct,D,E,F,G"</formula1>
     </dataValidation>
-    <dataValidation sqref="Y5:Y1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Please choose a value from the dropdown list." type="list" errorStyle="stop">
+    <dataValidation sqref="W5:W1000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Please choose a value from the dropdown list." type="list" errorStyle="stop">
       <formula1>"Trust,Usufruct,Pledge"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>